<commit_message>
GIC 2026 Blog added
</commit_message>
<xml_diff>
--- a/AI_INVOLVEMENT_LOG.xlsx
+++ b/AI_INVOLVEMENT_LOG.xlsx
@@ -254,9 +254,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -286,10 +283,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1132,10 +1128,10 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="2"/>
+      <c r="A31" s="1"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="2"/>
+      <c r="A32" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Formatting and css changes to last commit content
</commit_message>
<xml_diff>
--- a/AI_INVOLVEMENT_LOG.xlsx
+++ b/AI_INVOLVEMENT_LOG.xlsx
@@ -587,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1133,6 +1133,9 @@
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
     </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
IBO 2015 Added, minor security fixes, and more SEO improvements
</commit_message>
<xml_diff>
--- a/AI_INVOLVEMENT_LOG.xlsx
+++ b/AI_INVOLVEMENT_LOG.xlsx
@@ -254,6 +254,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -283,9 +286,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1136,6 +1140,12 @@
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
     </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>